<commit_message>
Dark mode + neutral A/B naming + side-aware diff colors
- Follow OS dark/light scheme: Fusion style + matching QPalette applied
  at startup, plus theme-aware diff color set (light & dark variants).
- Drop the 'antiguo/nuevo' framing: files are now A and B, with their
  basenames shown in headers, button labels, banners, status bar, and
  dirty markers. Collision between basenames disambiguates with parent
  folder. Long names are truncated with ellipsis.
- Side-aware diff coloring: when a cell exists on only one side, the
  side with content gets the 'present' tint and the other side gets a
  neutral 'absent' tint instead of both being painted the same colour.
  Communicates orphan cells like Beyond Compare / git.
- Window title becomes 'Excel Diff Tool'.
</commit_message>
<xml_diff>
--- a/ejemplos/antiguo.xlsx
+++ b/ejemplos/antiguo.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -491,10 +491,10 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="E2" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="F2" s="2">
         <f>D2*E2</f>
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="E4" t="n">
         <v>120</v>
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.1</v>
+        <v>2.4</v>
       </c>
       <c r="E5" t="n">
         <v>60</v>
@@ -690,7 +690,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -702,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -864,7 +863,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -876,7 +874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -928,7 +926,6 @@
         <v/>
       </c>
     </row>
-    <row r="5"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>